<commit_message>
updates to scripts to fix testing issues, and also to better handle location of config.env
</commit_message>
<xml_diff>
--- a/docs/malaria/catalogo_malaria.xlsx
+++ b/docs/malaria/catalogo_malaria.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catálogo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Catálogo" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -693,7 +693,7 @@
       </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>https://delphi-catalogo.example.org/malaria/mal_01.html</t>
+          <t>https://kaiserso.github.io/INS_delphi/malaria/mal_01.html</t>
         </is>
       </c>
     </row>
@@ -805,7 +805,7 @@
       </c>
       <c r="V3" s="3" t="inlineStr">
         <is>
-          <t>https://delphi-catalogo.example.org/malaria/mal_02.html</t>
+          <t>https://kaiserso.github.io/INS_delphi/malaria/mal_02.html</t>
         </is>
       </c>
     </row>
@@ -920,7 +920,7 @@
       </c>
       <c r="V4" s="2" t="inlineStr">
         <is>
-          <t>https://delphi-catalogo.example.org/malaria/mal_03.html</t>
+          <t>https://kaiserso.github.io/INS_delphi/malaria/mal_03.html</t>
         </is>
       </c>
     </row>
@@ -1028,7 +1028,7 @@
       </c>
       <c r="V5" s="3" t="inlineStr">
         <is>
-          <t>https://delphi-catalogo.example.org/malaria/mal_04.html</t>
+          <t>https://kaiserso.github.io/INS_delphi/malaria/mal_04.html</t>
         </is>
       </c>
     </row>
@@ -1149,7 +1149,7 @@
       </c>
       <c r="V6" s="2" t="inlineStr">
         <is>
-          <t>https://delphi-catalogo.example.org/malaria/mal_05.html</t>
+          <t>https://kaiserso.github.io/INS_delphi/malaria/mal_05.html</t>
         </is>
       </c>
     </row>
@@ -1259,7 +1259,7 @@
       </c>
       <c r="V7" s="3" t="inlineStr">
         <is>
-          <t>https://delphi-catalogo.example.org/malaria/mal_06.html</t>
+          <t>https://kaiserso.github.io/INS_delphi/malaria/mal_06.html</t>
         </is>
       </c>
     </row>
@@ -1367,7 +1367,7 @@
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="inlineStr">
         <is>
-          <t>https://delphi-catalogo.example.org/malaria/mal_07.html</t>
+          <t>https://kaiserso.github.io/INS_delphi/malaria/mal_07.html</t>
         </is>
       </c>
     </row>
@@ -1479,7 +1479,7 @@
       </c>
       <c r="V9" s="3" t="inlineStr">
         <is>
-          <t>https://delphi-catalogo.example.org/malaria/mal_08.html</t>
+          <t>https://kaiserso.github.io/INS_delphi/malaria/mal_08.html</t>
         </is>
       </c>
     </row>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="V10" s="2" t="inlineStr">
         <is>
-          <t>https://delphi-catalogo.example.org/malaria/mal_09.html</t>
+          <t>https://kaiserso.github.io/INS_delphi/malaria/mal_09.html</t>
         </is>
       </c>
     </row>
@@ -1703,7 +1703,7 @@
       </c>
       <c r="V11" s="3" t="inlineStr">
         <is>
-          <t>https://delphi-catalogo.example.org/malaria/mal_10.html</t>
+          <t>https://kaiserso.github.io/INS_delphi/malaria/mal_10.html</t>
         </is>
       </c>
     </row>
@@ -1815,7 +1815,7 @@
       </c>
       <c r="V12" s="2" t="inlineStr">
         <is>
-          <t>https://delphi-catalogo.example.org/malaria/mal_11.html</t>
+          <t>https://kaiserso.github.io/INS_delphi/malaria/mal_11.html</t>
         </is>
       </c>
     </row>
@@ -1928,7 +1928,7 @@
       </c>
       <c r="V13" s="3" t="inlineStr">
         <is>
-          <t>https://delphi-catalogo.example.org/malaria/mal_12.html</t>
+          <t>https://kaiserso.github.io/INS_delphi/malaria/mal_12.html</t>
         </is>
       </c>
     </row>
@@ -2040,7 +2040,7 @@
       </c>
       <c r="V14" s="2" t="inlineStr">
         <is>
-          <t>https://delphi-catalogo.example.org/malaria/mal_13.html</t>
+          <t>https://kaiserso.github.io/INS_delphi/malaria/mal_13.html</t>
         </is>
       </c>
     </row>
@@ -2150,7 +2150,7 @@
       </c>
       <c r="V15" s="3" t="inlineStr">
         <is>
-          <t>https://delphi-catalogo.example.org/malaria/mal_14.html</t>
+          <t>https://kaiserso.github.io/INS_delphi/malaria/mal_14.html</t>
         </is>
       </c>
     </row>
@@ -2267,7 +2267,7 @@
       </c>
       <c r="V16" s="2" t="inlineStr">
         <is>
-          <t>https://delphi-catalogo.example.org/malaria/mal_15.html</t>
+          <t>https://kaiserso.github.io/INS_delphi/malaria/mal_15.html</t>
         </is>
       </c>
     </row>
@@ -2379,7 +2379,7 @@
       </c>
       <c r="V17" s="3" t="inlineStr">
         <is>
-          <t>https://delphi-catalogo.example.org/malaria/mal_16.html</t>
+          <t>https://kaiserso.github.io/INS_delphi/malaria/mal_16.html</t>
         </is>
       </c>
     </row>
@@ -2473,7 +2473,7 @@
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="inlineStr">
         <is>
-          <t>https://delphi-catalogo.example.org/malaria/mal_17.html</t>
+          <t>https://kaiserso.github.io/INS_delphi/malaria/mal_17.html</t>
         </is>
       </c>
     </row>
@@ -2581,7 +2581,7 @@
       </c>
       <c r="V19" s="3" t="inlineStr">
         <is>
-          <t>https://delphi-catalogo.example.org/malaria/mal_18.html</t>
+          <t>https://kaiserso.github.io/INS_delphi/malaria/mal_18.html</t>
         </is>
       </c>
     </row>
@@ -2689,7 +2689,7 @@
       </c>
       <c r="V20" s="2" t="inlineStr">
         <is>
-          <t>https://delphi-catalogo.example.org/malaria/mal_19.html</t>
+          <t>https://kaiserso.github.io/INS_delphi/malaria/mal_19.html</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
pushed date/time stamp to first page to save a click, updated intervention labels to be more self-explanatory
</commit_message>
<xml_diff>
--- a/docs/malaria/catalogo_malaria.xlsx
+++ b/docs/malaria/catalogo_malaria.xlsx
@@ -832,7 +832,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Tratamento de casos (AL)</t>
+          <t>Tratamento de casos (Artemeter-Lumefantrine)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1394,7 +1394,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Distribuição de RTI (campanhas de acesso universal)</t>
+          <t>Distribuição de redes tratadas com insecticida (campanhas de acesso universal)</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -1404,7 +1404,7 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>As RTI  constituem a principal intervenção no controlo de vectores em Moçambique. A campanha de acesso universal é um método comprovadamente de rápido alcance e que permite uma alta e equitativa cobertura. Assume-se que a vida útil das RTIs varia de 2 a 3 anos, portanto, as campanhas massiva serão programadas tendo em conta esse periodo.</t>
+          <t>As redes tratadas com insecticida (RTI) constituem a principal intervenção no controlo de vectores em Moçambique. A campanha de acesso universal é um método comprovadamente de rápido alcance e que permite uma alta e equitativa cobertura. Assume-se que a vida útil das RTIs varia de 2 a 3 anos, portanto, as campanhas massiva serão programadas tendo em conta esse periodo.</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -1628,7 +1628,7 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>O TIP consiste na administração de um ciclo de tratamento de Sulfadoxina-pirimetamina (SP) em intervalos predeterminados, independentemente de a mulher grávida estar ou não infetada com malária. Esta intervenção será oferecida a partir das 13 semanas de gestação.</t>
+          <t>O tratamento intermitente preventivo (TIP) consiste na administração de um ciclo de tratamento de Sulfadoxina-pirimetamina (SP) em intervalos predeterminados, independentemente de a mulher grávida estar ou não infetada com malária. Esta intervenção será oferecida a partir das 13 semanas de gestação.</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
@@ -1730,7 +1730,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Distribuição de RTI nas CPNs</t>
+          <t>Distribuição de RTI nas consultas pré-natais (CPN)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1740,7 +1740,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>A distribuição de redes na CPN constitui um mecanismo de distribuição continua de redes fora das campanhas massivas , e é projectada para manter a cobertura alta de redes a nível da comunmidade, fornecendo redes as comunidades numa base regular. Nas CPNs as RTIs são entregues ás mulheres grávidas no primeiro contacto com a US (ª1 CPN).</t>
+          <t>A distribuição de redes na consulta pré-natal (CPN) constitui um mecanismo de distribuição continua de redes fora das campanhas massivas , e é projectada para manter a cobertura alta de redes a nível da comunmidade, fornecendo redes as comunidades numa base regular. Nas CPNs as RTIs são entregues ás mulheres grávidas no primeiro contacto com a US (ª1 CPN).</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Supervisão integrada e Avaliação de qualidade de dados usando  a plataforma SIIM</t>
+          <t>Supervisão integrada e Avaliação de qualidade de dados usando o Sistema Integrado de Informação da Malária (SIIM)</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">

</xml_diff>